<commit_message>
🔄 Index Monitor Update - 2026-09-09 07:03:28 UTC
Detected 21 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_evidence.xlsx
+++ b/index_changes_evidence.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -565,32 +565,32 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>TopBuild Corp</t>
+          <t>Synovus</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>BLD</t>
+          <t>SNV</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>IES Holdings</t>
+          <t>UiPath</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>IESC</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -600,12 +600,12 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: (NYSE: QXO ) is acquiring TopBuild in a deal expected to close soon, pending final closing conditions.</t>
+          <t>Merger/Acquisition: S&amp;P MidCap 400 constituent Pinnacle Financial Partners Inc. acquired Synovus Financial Corp.[17]</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/honeywell-aerospace-set-to-join-sp-500--sp-100-others-to-join-sp-midcap-400-and-sp-smallcap-600-302808386.html</t>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_400_companies</t>
         </is>
       </c>
     </row>
@@ -617,35 +617,47 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Masimo</t>
+          <t>Frontier Communications</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>MASI</t>
+          <t>FYBR</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>StandardAero</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>SARO</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Removed, no matching addition found</t>
+          <t>Same effective date</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: (NYSE: DHR ) is acquiring Masimo in a deal expected to be completed soon pending final conditions.</t>
+          <t>Merger/Acquisition: S&amp;P 500 &amp; S&amp;P 100 constituentVerizonCommunications Inc. acquired Frontier Communications Parent.[16]</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/sirius-xm-holdings-set-to-join-sp-midcap-400-302794483.html</t>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_400_companies</t>
         </is>
       </c>
     </row>
@@ -657,35 +669,47 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Chart Industries</t>
+          <t>Civitas Resources</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>GTLS</t>
+          <t>CIVI</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>TTM Technologies</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>TTMI</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Removed, no matching addition found</t>
+          <t>Same effective date</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: (NASD: BKR) is to acquire Chart Industries in a deal expected to close July 16, pending final closing conditions.</t>
+          <t>Merger/Acquisition: S&amp;P SmallCap 600 constituentSM EnergyCompany acquired Civitas Resources.[15]</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/brightspring-health-services-set-to-join-sp-midcap-400-and-karman-holdings-to-join-sp-smallcap-600-302825665.html</t>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_400_companies</t>
         </is>
       </c>
     </row>
@@ -697,35 +721,47 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>National Storage Affiliates Trust</t>
+          <t>Cadence Bank</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>NSA</t>
+          <t>CADE</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Advanced Energy</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>AEIS</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Removed, no matching addition found</t>
+          <t>Same effective date</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo...</t>
+          <t>Merger/Acquisition: S&amp;P 500 constituentFifth Third Bancorpacquired Comerica.[15] | Merger/Acquisition: S&amp;P 500 constituentHuntington BancsharesInc. acquired Cadence Bank.[15]</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/molina-healthcare-set-to-join-sp-midcap-400-and-construction-partners-to-join-sp-smallcap-600-302828046.html</t>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_400_companies</t>
         </is>
       </c>
     </row>
@@ -737,35 +773,47 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Taylor Morrison Home</t>
+          <t>Comerica</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>TMHC</t>
+          <t>CMA</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>American Healthcare REIT</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>AHR</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Removed, no matching addition found</t>
+          <t>Same effective date</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: (NYSE: BRK.A /BRK.B) is acquiring Taylor Morrison Home in a deal expected to close on or about that date, pending final closing conditions.</t>
+          <t>Merger/Acquisition: S&amp;P 500 constituentHuntington BancsharesInc. acquired Cadence Bank.[15] | Merger/Acquisition: S&amp;P 500 constituentFifth Third Bancorpacquired Comerica.[15]</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/krystal-biotech-set-to-join-sp-midcap-400-tutor-perini-and-v2x-to-join-sp-smallcap-600-302830022.html</t>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_400_companies</t>
         </is>
       </c>
     </row>
@@ -777,82 +825,94 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Webster Financial</t>
+          <t>PotlatchDeltic</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>WBS</t>
+          <t>PCH</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Dutch Bros Inc.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>BROS</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Removed, no matching addition found</t>
+          <t>Same effective date</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: (BMEX /NYSE: SAN ) is acquiring Webster Financial in a deal expected to be completed soon pending final conditions.</t>
+          <t>Merger/Acquisition: S&amp;P MidCap 400 constituent Rayonier Inc. acquired PotlatchDeltic.[15]</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/reddit-set-to-join-sp-500-and-sun-communities-to-join-sp-midcap-400-302851432.html</t>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_400_companies</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 500</t>
+          <t>S&amp;P 400</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>TopBuild Corp</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>EA</t>
+          <t>BLD</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Honeywell Aerospace</t>
+          <t>IES Holdings</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>HONA</t>
+          <t>IESC</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Different effective dates — paired for reference only</t>
+          <t>Same effective date</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Spin-off: Post spin-off Honeywell International will be renamed Honeywell Technologies Inc. | Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo...</t>
+          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: (NYSE: QXO ) is acquiring TopBuild in a deal expected to close soon, pending final closing conditions.</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
@@ -864,22 +924,22 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 500</t>
+          <t>S&amp;P 400</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>AvalonBay Communities</t>
+          <t>Masimo</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>AVB</t>
+          <t>MASI</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
@@ -892,34 +952,34 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: S&amp;P 500 constituent Equity Residential (NYSE: EQR ) is acquiring AvalonBay Communities in a deal expected to be completed soon, pending final conditions.</t>
+          <t>Merger/Acquisition: (NYSE: DHR ) is acquiring Masimo in a deal expected to be completed soon pending final conditions.</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/reddit-set-to-join-sp-500-and-sun-communities-to-join-sp-midcap-400-302851432.html</t>
+          <t>https://www.prnewswire.com/news-releases/sirius-xm-holdings-set-to-join-sp-midcap-400-302794483.html</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 500</t>
+          <t>S&amp;P 400</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>The Trade Desk</t>
+          <t>Chart Industries</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>TTD</t>
+          <t>GTLS</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
@@ -932,205 +992,169 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo...</t>
+          <t>Merger/Acquisition: (NASD: BKR) is to acquire Chart Industries in a deal expected to close July 16, pending final closing conditions.</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+          <t>https://www.prnewswire.com/news-releases/brightspring-health-services-set-to-join-sp-midcap-400-and-karman-holdings-to-join-sp-smallcap-600-302825665.html</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 600</t>
+          <t>S&amp;P 400</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Kennedy-Wilson Holdings</t>
+          <t>National Storage Affiliates Trust</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>KW</t>
+          <t>NSA</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>National Health Investors</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>NHI</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Different effective dates — paired for reference only</t>
+          <t>Removed, no matching addition found</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: A consortium led by KW's CEO with Fairfax Financial Holdings Limited (TSE: FFH) is acquiring Kennedy-Wilson Holdings in a deal expected to close soon, pending final closing conditions.</t>
+          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo...</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/honeywell-aerospace-set-to-join-sp-500--sp-100-others-to-join-sp-midcap-400-and-sp-smallcap-600-302808386.html</t>
+          <t>https://www.prnewswire.com/news-releases/molina-healthcare-set-to-join-sp-midcap-400-and-construction-partners-to-join-sp-smallcap-600-302828046.html</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 600</t>
+          <t>S&amp;P 400</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>ProAssurance</t>
+          <t>Taylor Morrison Home</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>PRA</t>
+          <t>TMHC</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Construction Partners</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>ROAD</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Different effective dates — paired for reference only</t>
+          <t>Removed, no matching addition found</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: The Doctors Company is acquiring ProAssurance in a cash deal expected to close soon, pending final closing conditions.</t>
+          <t>Merger/Acquisition: (NYSE: BRK.A /BRK.B) is acquiring Taylor Morrison Home in a deal expected to close on or about that date, pending final closing conditions.</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/molina-healthcare-set-to-join-sp-midcap-400-and-construction-partners-to-join-sp-smallcap-600-302828046.html</t>
+          <t>https://www.prnewswire.com/news-releases/krystal-biotech-set-to-join-sp-midcap-400-tutor-perini-and-v2x-to-join-sp-smallcap-600-302830022.html</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 600</t>
+          <t>S&amp;P 400</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Select Medical Holdings</t>
+          <t>Webster Financial</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>SEM</t>
+          <t>WBS</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>ADI Global Distribution</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>ADIG</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-04</t>
-        </is>
-      </c>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Different effective dates — paired for reference only</t>
+          <t>Removed, no matching addition found</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: Select Medical Holdings is being acquired in a deal expected to be completed soon, pending final closing conditions.</t>
+          <t>Merger/Acquisition: (BMEX /NYSE: SAN ) is acquiring Webster Financial in a deal expected to be completed soon pending final conditions.</t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/ferguson-enterprises-set-to-join-sp-500-and-adi-global-distribution-to-join-sp-smallcap-600-302840407.html</t>
+          <t>https://www.prnewswire.com/news-releases/reddit-set-to-join-sp-500-and-sun-communities-to-join-sp-midcap-400-302851432.html</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 600</t>
+          <t>S&amp;P 500</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Stellar Bancorp</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>STEL</t>
+          <t>EA</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>The Trade Desk</t>
+          <t>Honeywell Aerospace</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>TTD</t>
+          <t>HONA</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1140,34 +1164,34 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: (NYSE: PB ) is acquiring Stellar Bancorp in a deal expected to close July 1.</t>
+          <t>Spin-off: Post spin-off Honeywell International will be renamed Honeywell Technologies Inc. | Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo...</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+          <t>https://www.prnewswire.com/news-releases/honeywell-aerospace-set-to-join-sp-500--sp-100-others-to-join-sp-midcap-400-and-sp-smallcap-600-302808386.html</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 600</t>
+          <t>S&amp;P 500</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Whitestone REIT</t>
+          <t>AvalonBay Communities</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>WSR</t>
+          <t>AVB</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
@@ -1180,34 +1204,34 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: (NYSE: ARES ) is acquiring Whitestone REIT in a deal expected to close on or about that date, pending final closing conditions.</t>
+          <t>Merger/Acquisition: S&amp;P 500 constituent Equity Residential (NYSE: EQR ) is acquiring AvalonBay Communities in a deal expected to be completed soon, pending final conditions.</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/midera-food-processing-and-centrus-energy-set-to-join-sp-smallcap-600-302817273.html</t>
+          <t>https://www.prnewswire.com/news-releases/reddit-set-to-join-sp-500-and-sun-communities-to-join-sp-midcap-400-302851432.html</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 600</t>
+          <t>S&amp;P 500</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Catalyst Pharmaceuticals</t>
+          <t>The Trade Desk</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>CPRX</t>
+          <t>TTD</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
@@ -1220,12 +1244,12 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: is acquiring Catalyst Pharmaceuticals in a deal expected to close soon, pending final closing conditions.</t>
+          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo...</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/solaris-energy-infrastructure-set-to-join-sp-smallcap-600-302822362.html</t>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
         </is>
       </c>
     </row>
@@ -1237,35 +1261,47 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Avanos Medical</t>
+          <t>Brandywine Realty Trust</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>AVNS</t>
+          <t>BDN</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr"/>
-      <c r="G18" s="2" t="inlineStr"/>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Versant Media Group</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>VSNT</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Removed, no matching addition found</t>
+          <t>Same effective date</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: American Industrial Partners is acquiring Avanos Medical in a deal expected to close soon, pending final closing conditions.</t>
+          <t>Spin-off: VSNT was spun off fromComcastand replaced BDN which was no longer representative of the small-cap market space.[38]</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/krystal-biotech-set-to-join-sp-midcap-400-tutor-perini-and-v2x-to-join-sp-smallcap-600-302830022.html</t>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
         </is>
       </c>
     </row>
@@ -1277,35 +1313,47 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Two Harbors Investment</t>
+          <t>Guess, Inc.</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>TWO</t>
+          <t>GES</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" s="2" t="inlineStr"/>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Winmark</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>WINA</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Removed, no matching addition found</t>
+          <t>Same effective date</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo...</t>
+          <t>Merger/Acquisition: WINA replaced GES after it was acquired byAuthentic Brands Groupand the Rolling Stockholders.[37]</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/five9-set-to-join-sp-smallcap-600-302838329.html</t>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
         </is>
       </c>
     </row>
@@ -1317,33 +1365,1585 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
+          <t>TTM Technologies</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>TTMI</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Amneal Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>AMRX</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: AMRX replaced TTMI, which replaced Civitas Resources in theS&amp;P 400after it was acquired bySM Energy.[36]</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Advanced Energy</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>AEIS</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Apellis Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>APLS</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: APLS replaced AEIS, which replacedComericain the S&amp;P 400 after it was acquired byFifth Third Bank.[36]</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Dynavax Technologies</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>DVAX</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>OneSpaWorld Holdings</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>OSW</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: OSW replaced DVAX after it was acquired bySanofi.[35]</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>TreeHouse Foods</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>THS</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Merchants Bancorp</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>MBIN</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: MBIN replaced THS after it was acquired by Investindustrial S.A.[34]</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Hillenbrand</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>HI</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>RingCentral</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>RNG</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: RNG replaced HI after it was acquired byLone Star Funds.[33]</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Alexander &amp; Baldwin</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>ALEX</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Napco Security Technologies</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>NSSC</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: NSSC replaced ALEX after it was acquired by an investor group comprising MW Group and funds affiliated with DivcoWest andBlackstone Real Estate.[32]</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Tegna Inc.</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>TGNA</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Vita Coco</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>COCO</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: COCO replaced TGNA after it was acquired byNexstar Media Group.[31]</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Titan International, Inc.</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>TWI</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Versigent</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>VGNT</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Spin-off: VGNT was spun off fromAptivand replaced TWI which was no longer representative of the small-cap market space.[30]</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Air Lease Corporation</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Atmus Filtration Technologies</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>ATMU</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: ATMU replaced AL after it was acquired bySumitomo Corporation.[29]</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Sealed Air</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>SEE</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Diebold Nixdorf</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>DBD</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: DBD replaced SEE after it was acquired byClayton, Dubilier &amp; Rice.[27]</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Golden Entertainment</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>GDEN</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Lifestance Health</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>LFST</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: LFST replaced GDEN after it was acquired byVici PropertiesandBlake L. Sartini.[25]</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Apellis Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>APLS</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Alignment Healthcare</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>ALHC</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: ALHC replaced SNCY after it was acquired byAllegiant Travel Company.[22] | Merger/Acquisition: RELY replaced APLS after it was acquired byBiogen.[23]</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Sun Country Airlines</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>SNCY</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Bright Horizons</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>BFAM</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: BFAM replaced TPH after it was acquired bySumitomo Forestry.[23] | Merger/Acquisition: ALHC replaced SNCY after it was acquired byAllegiant Travel Company.[22]</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Tri Pointe Homes</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>TPH</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Remitly</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>RELY</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: RELY replaced APLS after it was acquired byBiogen.[23] | Merger/Acquisition: BFAM replaced TPH after it was acquired bySumitomo Forestry.[23]</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>CSG Systems</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>CSGS</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Flowers Foods</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>FLO</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: FLO replaced CSGS after it was acquired byNEC.[21]</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Enviri</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>NVRI</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Peloton Interactive</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>PTON</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Spin-off: PTON replaced NVRI after it spun off assets into a new publicly traded company. The new publicly traded company was not representative of the small-cap market space.[20]</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Mister Car Wash</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>MCW</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>F&amp;G</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>FG</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: FG replaced MCW after it was acquired byLeonard Green &amp; Partners.[21]</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Veris Residential</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>VRE</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Universal Technical Institute</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>UTI</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: UTI replaced VRE after it was acquired by Affinius Capital and Vista Hill Partners.[20]</t>
+        </is>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>American Woodmark</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>AMWD</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Dave</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>DAVE</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: DAVE replaced AMWD after it was acquired by MasterBrand Inc.[19]</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Shutterstock</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>SSTK</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>EPAM Systems</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>EPAM</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: EPAM was moved from theS&amp;P 500as it was more representative of the small cap market space. SSTK was removed from theS&amp;P 600as it was merged withGetty Images.[19]</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Core Laboratories</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>CLB</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Mobility Global</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>MBGL</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Spin-off: MBGL was spun off fromS&amp;P Globaland replaced CLB which was no longer representative of the small-cap market space.[13]</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Whitestone REIT</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>WSR</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Centrus Energy</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>LEU</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: LEU replaced WSR after it was acquired byAres Management.[11]</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Hertz Global Holdings</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>HTZ</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>ADI Global Distribution</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>ADIG</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Spin-off: ADIG was spun off fromResideoand replaced HTZ which was no longer representative of the small-cap market space.[5]</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/ferguson-enterprises-set-to-join-sp-500-and-adi-global-distribution-to-join-sp-smallcap-600-302840407.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Kennedy-Wilson Holdings</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>KW</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>National Health Investors</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>NHI</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Different effective dates — paired for reference only</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: A consortium led by KW's CEO with Fairfax Financial Holdings Limited (TSE: FFH) is acquiring Kennedy-Wilson Holdings in a deal expected to close soon, pending final closing conditions.</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/honeywell-aerospace-set-to-join-sp-500--sp-100-others-to-join-sp-midcap-400-and-sp-smallcap-600-302808386.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>ProAssurance</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>PRA</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Construction Partners</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>ROAD</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Different effective dates — paired for reference only</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: The Doctors Company is acquiring ProAssurance in a cash deal expected to close soon, pending final closing conditions.</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/molina-healthcare-set-to-join-sp-midcap-400-and-construction-partners-to-join-sp-smallcap-600-302828046.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Select Medical Holdings</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>SEM</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>The Trade Desk</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>TTD</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Different effective dates — paired for reference only</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: Select Medical Holdings is being acquired in a deal expected to be completed soon, pending final closing conditions.</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Stellar Bancorp</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>STEL</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="2" t="inlineStr"/>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Removed, no matching addition found</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: (NYSE: PB ) is acquiring Stellar Bancorp in a deal expected to close July 1.</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/allison-transmission-holdings-set-to-join-sp-midcap-400-and-goodyear-tire--rubber-to-join-sp-smallcap-600-302815143.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Whitestone REIT</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>WSR</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr"/>
+      <c r="F47" s="2" t="inlineStr"/>
+      <c r="G47" s="2" t="inlineStr"/>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Removed, no matching addition found</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: (NYSE: ARES ) is acquiring Whitestone REIT in a deal expected to close on or about that date, pending final closing conditions.</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/midera-food-processing-and-centrus-energy-set-to-join-sp-smallcap-600-302817273.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Catalyst Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>CPRX</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr"/>
+      <c r="G48" s="2" t="inlineStr"/>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Removed, no matching addition found</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: is acquiring Catalyst Pharmaceuticals in a deal expected to close soon, pending final closing conditions.</t>
+        </is>
+      </c>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/solaris-energy-infrastructure-set-to-join-sp-smallcap-600-302822362.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Avanos Medical</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>AVNS</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr"/>
+      <c r="F49" s="2" t="inlineStr"/>
+      <c r="G49" s="2" t="inlineStr"/>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>Removed, no matching addition found</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: American Industrial Partners is acquiring Avanos Medical in a deal expected to close soon, pending final closing conditions.</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/krystal-biotech-set-to-join-sp-midcap-400-tutor-perini-and-v2x-to-join-sp-smallcap-600-302830022.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Two Harbors Investment</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>TWO</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr"/>
+      <c r="G50" s="2" t="inlineStr"/>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Removed, no matching addition found</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo...</t>
+        </is>
+      </c>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/five9-set-to-join-sp-smallcap-600-302838329.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
           <t>Leggett &amp; Platt</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>LEG</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr"/>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr"/>
+      <c r="F51" s="2" t="inlineStr"/>
+      <c r="G51" s="2" t="inlineStr"/>
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>Removed, no matching addition found</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="I51" s="2" t="inlineStr">
         <is>
           <t>Merger/Acquisition: (NYSE: SGI ) is acquiring Leggett &amp; Platt in a deal expected to be completed soon, pending final closing conditions.</t>
         </is>
       </c>
-      <c r="J20" s="3" t="inlineStr">
+      <c r="J51" s="3" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/tenable-holdings-set-to-join-sp-smallcap-600-302861023.html</t>
         </is>
@@ -1370,6 +2970,37 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>